<commit_message>
feat: reconcile git with live Vercel state, ship broadband cost calculator
- Commit the 16-page content-gap pipeline batch (6 guides, 2 provider
  comparisons, 8 postcode city hubs) that was previously deployed straight
  from disk via `vercel --prod` without ever being committed — closes the
  git/production divergence flagged as the top item in the build tracker
- Add /tools/broadband-cost-calculator: true monthly cost + cost-per-Mbps
  calculator (components/BroadbandCostCalculator.tsx), validated via
  npm run build and a local render check before commit
- Add scripts/build_master_tracker.py: unified, priority-ranked Excel
  tracker across page builds and feature/UX builds, with status preserved
  across re-runs
- Add scripts/scrape_competitor_landscape.py and its research output,
  informing the growth playbook this batch also implements against

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/broadbandpicker-keyword-mapping.xlsx
+++ b/docs/broadbandpicker-keyword-mapping.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Keyword Mapping'!$A$1:$M$142</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Current Page Inventory'!$A$1:$H$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Current Page Inventory'!$A$1:$H$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Content Gap Roadmap'!$A$1:$N$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cluster Summary'!$A$1:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Methodology'!$A$1:$B$10</definedName>
@@ -198,8 +198,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CurrentPageInventoryTable" displayName="CurrentPageInventoryTable" ref="A1:H78" headerRowCount="1">
-  <autoFilter ref="A1:H78"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CurrentPageInventoryTable" displayName="CurrentPageInventoryTable" ref="A1:H79" headerRowCount="1">
+  <autoFilter ref="A1:H79"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Path"/>
     <tableColumn id="2" name="Topic Cluster"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>None supplied</t>
+          <t>https://docs.google.com/spreadsheets/d/1_IeyaXe1fSbXmV8Z4MdVOigMIz-cgK2h/edit</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Build the first non-complete page on Content Gap Roadmap. Each online run checks the live sitemap and HTTP response, moves completed pages below the active queue, labels their deployment status and strikes them through.</t>
+          <t>The standard production command builds up to five active pages from the top of the Content Gap Roadmap, one at a time. After each page it checks the live sitemap and HTTP response, moves completed pages below the active queue, labels their deployment status and strikes them through.</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Content gap — recommend new page</t>
+          <t>Existing page</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -8841,7 +8841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -8851,7 +8851,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -8914,13 +8914,19 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>broadband</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: / (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed to resolve</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -8940,13 +8946,19 @@
       </c>
       <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>broadband deals, best broadband deals, cheap broadband deals, uk broadband deals</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /deals (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed to re</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -8966,13 +8978,19 @@
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>compare broadband deals, compare broadband providers, broadband comparison uk</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /compare (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed to </t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -8992,13 +9010,19 @@
       </c>
       <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>broadband providers</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed t</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -9018,9 +9042,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): </t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -9040,9 +9070,15 @@
       </c>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed to r</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -9062,13 +9098,19 @@
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>broadband speed test, check my broadband speed</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /speed-test (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed </t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -9088,13 +9130,19 @@
       </c>
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>broadband glossary terms explained, what is fttp broadband, what is a good broadband speed</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /broadband-glossary (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443):</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -9114,9 +9162,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /about (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed to re</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -9136,9 +9190,15 @@
       </c>
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /contact (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed to </t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -9158,13 +9218,19 @@
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>how we make money broadband picker</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /how-we-make-money (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): </t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -9184,9 +9250,15 @@
       </c>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /how-we-review-broadband (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -9206,9 +9278,15 @@
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /editorial-policy (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): F</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -9228,9 +9306,15 @@
       </c>
       <c r="D15" s="3" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /privacy-policy (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Fai</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -9250,9 +9334,15 @@
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /cookie-policy (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Fail</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -9272,9 +9362,15 @@
       </c>
       <c r="D17" s="3" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /terms (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed to re</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -9294,13 +9390,19 @@
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>broadband providers for my area, broadband in my area, broadband postcode checker</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /postcode (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Failed to</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -9320,75 +9422,93 @@
       </c>
       <c r="D19" s="3" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
           <t>broadband providers london, best broadband london</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /postcode/london (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Fa</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>/research/uk-broadband-customer-satisfaction</t>
+          <t>/postcode/bristol</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Trust &amp; research</t>
+          <t>Postcode &amp; location</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Research dashboard</t>
+          <t>City hub</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>uk broadband customer satisfaction</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>broadband providers bristol</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /postcode/bristol (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): F</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>/guides/best-business-broadband-providers-uk</t>
+          <t>/research/uk-broadband-customer-satisfaction</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Business broadband</t>
+          <t>Trust &amp; research</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Guide</t>
+          <t>Research dashboard</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>best business broadband providers uk, business broadband providers</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
+          <t>uk broadband customer satisfaction</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /research/uk-broadband-customer-satisfaction (Caused by NameResolutionError("HTTPSConnection(host='broadband</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>/guides/best-phone-and-broadband-deals</t>
+          <t>/guides/best-business-broadband-providers-uk</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Phone &amp; bundles</t>
+          <t>Business broadband</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -9398,23 +9518,29 @@
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>phone and broadband deals, landline broadband deals</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>best business broadband providers uk, business broadband providers</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-business-broadband-providers-uk (Caused by NameResolutionError("HTTPSConnection(host='broadband</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>/guides/satellite-broadband-uk</t>
+          <t>/guides/best-phone-and-broadband-deals</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Alternative access</t>
+          <t>Phone &amp; bundles</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -9424,44 +9550,56 @@
       </c>
       <c r="D23" s="3" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>satellite broadband uk</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
+          <t>phone and broadband deals, landline broadband deals</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-phone-and-broadband-deals (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>/providers/bt</t>
+          <t>/guides/satellite-broadband-uk</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Provider brand</t>
+          <t>Alternative access</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Provider page</t>
+          <t>Guide</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>bt broadband, bt broadband deals, bt broadband reviews</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>satellite broadband uk</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/satellite-broadband-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk',</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>/providers/sky</t>
+          <t>/providers/bt</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -9476,18 +9614,24 @@
       </c>
       <c r="D25" s="3" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>sky broadband, sky broadband deals, sky broadband reviews</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
+          <t>bt broadband, bt broadband deals, bt broadband reviews</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/bt (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Faile</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>/providers/virgin-media</t>
+          <t>/providers/sky</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -9502,18 +9646,24 @@
       </c>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>virgin media broadband, virgin media broadband deals, virgin media broadband reviews</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
+          <t>sky broadband, sky broadband deals, sky broadband reviews</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/sky (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Fail</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>/providers/ee</t>
+          <t>/providers/virgin-media</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -9528,18 +9678,24 @@
       </c>
       <c r="D27" s="3" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>ee broadband, ee broadband deals, ee broadband reviews</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
+          <t>virgin media broadband, virgin media broadband deals, virgin media broadband reviews</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/virgin-media (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=4</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>/providers/talktalk</t>
+          <t>/providers/ee</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -9554,18 +9710,24 @@
       </c>
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>talktalk broadband, talktalk broadband deals, talktalk broadband reviews</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
+          <t>ee broadband, ee broadband deals, ee broadband reviews</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/ee (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Faile</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>/providers/plusnet</t>
+          <t>/providers/talktalk</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -9580,18 +9742,24 @@
       </c>
       <c r="D29" s="3" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>plusnet broadband, plusnet broadband deals, plusnet broadband reviews</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
+          <t>talktalk broadband, talktalk broadband deals, talktalk broadband reviews</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/talktalk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443):</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>/providers/vodafone</t>
+          <t>/providers/plusnet</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -9606,18 +9774,24 @@
       </c>
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>vodafone broadband, vodafone broadband deals, vodafone broadband reviews</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
+          <t>plusnet broadband, plusnet broadband deals, plusnet broadband reviews</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/plusnet (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): </t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>/providers/now-broadband</t>
+          <t>/providers/vodafone</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -9632,18 +9806,24 @@
       </c>
       <c r="D31" s="3" t="inlineStr"/>
       <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>now broadband broadband, now broadband broadband deals, now broadband broadband reviews</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr"/>
+          <t>vodafone broadband, vodafone broadband deals, vodafone broadband reviews</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/vodafone (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443):</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>/providers/hyperoptic</t>
+          <t>/providers/now-broadband</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -9658,18 +9838,24 @@
       </c>
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>hyperoptic broadband, hyperoptic broadband deals, hyperoptic broadband reviews</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
+          <t>now broadband broadband, now broadband broadband deals, now broadband broadband reviews</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/now-broadband (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>/providers/community-fibre</t>
+          <t>/providers/hyperoptic</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -9684,18 +9870,24 @@
       </c>
       <c r="D33" s="3" t="inlineStr"/>
       <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>community fibre broadband, community fibre broadband deals, community fibre broadband reviews</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr"/>
+          <t>hyperoptic broadband, hyperoptic broadband deals, hyperoptic broadband reviews</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/hyperoptic (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>/providers/zen-internet</t>
+          <t>/providers/community-fibre</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -9710,18 +9902,24 @@
       </c>
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>zen internet broadband, zen internet broadband deals, zen internet broadband reviews</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr"/>
+          <t>community fibre broadband, community fibre broadband deals, community fibre broadband reviews</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/community-fibre (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', por</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>/providers/toob</t>
+          <t>/providers/zen-internet</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -9736,44 +9934,56 @@
       </c>
       <c r="D35" s="3" t="inlineStr"/>
       <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>toob broadband, toob broadband deals, toob broadband reviews</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr"/>
+          <t>zen internet broadband, zen internet broadband deals, zen internet broadband reviews</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/zen-internet (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=4</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>/providers/compare/bt-vs-sky</t>
+          <t>/providers/toob</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Provider vs comparison</t>
+          <t>Provider brand</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Comparison page</t>
+          <t>Provider page</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>bt vs sky broadband</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr"/>
+          <t>toob broadband, toob broadband deals, toob broadband reviews</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/toob (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', port=443): Fai</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>/providers/compare/bt-vs-virgin-media</t>
+          <t>/providers/compare/bt-vs-sky</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -9788,18 +9998,24 @@
       </c>
       <c r="D37" s="3" t="inlineStr"/>
       <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>bt vs virgin media broadband</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
+          <t>bt vs sky broadband</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/bt-vs-sky (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', p</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>/providers/compare/sky-vs-vodafone</t>
+          <t>/providers/compare/bt-vs-virgin-media</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -9814,18 +10030,24 @@
       </c>
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>sky vs vodafone broadband</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr"/>
+          <t>bt vs virgin media broadband</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/bt-vs-virgin-media (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>/providers/compare/ee-vs-bt</t>
+          <t>/providers/compare/sky-vs-vodafone</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -9840,18 +10062,24 @@
       </c>
       <c r="D39" s="3" t="inlineStr"/>
       <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>ee vs bt broadband</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr"/>
+          <t>sky vs vodafone broadband</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/sky-vs-vodafone (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>/providers/compare/talktalk-vs-now-broadband</t>
+          <t>/providers/compare/ee-vs-bt</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -9866,18 +10094,24 @@
       </c>
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>talktalk vs now broadband</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
+          <t>ee vs bt broadband</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/ee-vs-bt (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', po</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>/providers/compare/virgin-media-vs-vodafone</t>
+          <t>/providers/compare/talktalk-vs-now-broadband</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -9892,18 +10126,24 @@
       </c>
       <c r="D41" s="3" t="inlineStr"/>
       <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>virgin media vs vodafone broadband</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr"/>
+          <t>talktalk vs now broadband</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/talktalk-vs-now-broadband (Caused by NameResolutionError("HTTPSConnection(host='broadband</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>/providers/compare/sky-vs-virgin-media</t>
+          <t>/providers/compare/virgin-media-vs-vodafone</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -9918,18 +10158,24 @@
       </c>
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>sky vs virgin media broadband</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
+          <t>virgin media vs vodafone broadband</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/virgin-media-vs-vodafone (Caused by NameResolutionError("HTTPSConnection(host='broadbandp</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>/providers/compare/hyperoptic-vs-community-fibre</t>
+          <t>/providers/compare/sky-vs-virgin-media</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -9944,18 +10190,24 @@
       </c>
       <c r="D43" s="3" t="inlineStr"/>
       <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>hyperoptic vs community fibre</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr"/>
+          <t>sky vs virgin media broadband</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/sky-vs-virgin-media (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>/providers/compare/bt-vs-vodafone</t>
+          <t>/providers/compare/hyperoptic-vs-community-fibre</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -9970,18 +10222,24 @@
       </c>
       <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>bt vs vodafone broadband</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr"/>
+          <t>hyperoptic vs community fibre</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/hyperoptic-vs-community-fibre (Caused by NameResolutionError("HTTPSConnection(host='broad</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>/providers/compare/ee-vs-sky</t>
+          <t>/providers/compare/bt-vs-vodafone</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -9996,18 +10254,24 @@
       </c>
       <c r="D45" s="3" t="inlineStr"/>
       <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>ee vs sky broadband</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr"/>
+          <t>bt vs vodafone broadband</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/bt-vs-vodafone (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.u</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>/providers/compare/bt-vs-talktalk</t>
+          <t>/providers/compare/ee-vs-sky</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -10022,18 +10286,24 @@
       </c>
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>bt vs talktalk broadband</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr"/>
+          <t>ee vs sky broadband</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/ee-vs-sky (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', p</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>/providers/compare/ee-vs-vodafone</t>
+          <t>/providers/compare/bt-vs-talktalk</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -10048,18 +10318,24 @@
       </c>
       <c r="D47" s="3" t="inlineStr"/>
       <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>ee vs vodafone broadband</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr"/>
+          <t>bt vs talktalk broadband</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/bt-vs-talktalk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.u</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>/providers/compare/sky-vs-talktalk</t>
+          <t>/providers/compare/ee-vs-vodafone</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -10074,18 +10350,24 @@
       </c>
       <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>sky vs talktalk broadband</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr"/>
+          <t>ee vs vodafone broadband</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/ee-vs-vodafone (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.u</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>/providers/compare/plusnet-vs-bt</t>
+          <t>/providers/compare/sky-vs-talktalk</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -10100,18 +10382,24 @@
       </c>
       <c r="D49" s="3" t="inlineStr"/>
       <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>plusnet vs bt broadband</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr"/>
+          <t>sky vs talktalk broadband</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/sky-vs-talktalk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>/providers/compare/plusnet-vs-sky</t>
+          <t>/providers/compare/plusnet-vs-bt</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -10126,18 +10414,24 @@
       </c>
       <c r="D50" s="2" t="inlineStr"/>
       <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>plusnet vs sky broadband</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr"/>
+          <t>plusnet vs bt broadband</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/plusnet-vs-bt (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>/providers/compare/vodafone-vs-talktalk</t>
+          <t>/providers/compare/plusnet-vs-sky</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -10152,44 +10446,56 @@
       </c>
       <c r="D51" s="3" t="inlineStr"/>
       <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>vodafone vs talktalk broadband</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr"/>
+          <t>plusnet vs sky broadband</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/plusnet-vs-sky (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.u</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>/guides/how-to-switch-broadband-uk</t>
+          <t>/providers/compare/vodafone-vs-talktalk</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Editorial guide</t>
+          <t>Provider vs comparison</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Guide</t>
+          <t>Comparison page</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr"/>
       <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>switch broadband provider, how to switch broadband provider uk</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr"/>
+          <t>vodafone vs talktalk broadband</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /providers/compare/vodafone-vs-talktalk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicke</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>/guides/best-broadband-deals-uk</t>
+          <t>/guides/how-to-switch-broadband-uk</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -10204,14 +10510,24 @@
       </c>
       <c r="D53" s="3" t="inlineStr"/>
       <c r="E53" s="3" t="inlineStr"/>
-      <c r="F53" s="3" t="inlineStr"/>
-      <c r="G53" s="3" t="inlineStr"/>
-      <c r="H53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>switch broadband provider, how to switch broadband provider uk</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/how-to-switch-broadband-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>/guides/broadband-deals-with-no-mid-contract-price-rise</t>
+          <t>/guides/best-broadband-deals-uk</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -10226,18 +10542,20 @@
       </c>
       <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>broadband deals with no mid contract price rise</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-broadband-deals-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk'</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>/guides/best-broadband-and-tv-deals</t>
+          <t>/guides/broadband-deals-with-no-mid-contract-price-rise</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -10252,18 +10570,24 @@
       </c>
       <c r="D55" s="3" t="inlineStr"/>
       <c r="E55" s="3" t="inlineStr"/>
-      <c r="F55" s="3" t="inlineStr"/>
+      <c r="F55" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>best broadband and tv deals</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr"/>
+          <t>broadband deals with no mid contract price rise</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-deals-with-no-mid-contract-price-rise (Caused by NameResolutionError("HTTPSConnection(host</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>/guides/broadband-deals-under-20</t>
+          <t>/guides/best-broadband-and-tv-deals</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -10278,18 +10602,24 @@
       </c>
       <c r="D56" s="2" t="inlineStr"/>
       <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>broadband deals under 20, broadband deals under 20 a month</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr"/>
+          <t>best broadband and tv deals</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-broadband-and-tv-deals (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>/guides/broadband-deals-with-cashback</t>
+          <t>/guides/broadband-deals-under-20</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -10304,18 +10634,24 @@
       </c>
       <c r="D57" s="3" t="inlineStr"/>
       <c r="E57" s="3" t="inlineStr"/>
-      <c r="F57" s="3" t="inlineStr"/>
+      <c r="F57" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>broadband deals with cashback</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr"/>
+          <t>broadband deals under 20, broadband deals under 20 a month</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-deals-under-20 (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>/guides/broadband-deals-with-no-setup-fee</t>
+          <t>/guides/broadband-deals-with-cashback</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -10330,18 +10666,24 @@
       </c>
       <c r="D58" s="2" t="inlineStr"/>
       <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>broadband deals with no setup fee</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr"/>
+          <t>broadband deals with cashback</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-deals-with-cashback (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>/guides/best-rolling-monthly-broadband-deals</t>
+          <t>/guides/broadband-deals-with-no-setup-fee</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -10356,18 +10698,24 @@
       </c>
       <c r="D59" s="3" t="inlineStr"/>
       <c r="E59" s="3" t="inlineStr"/>
-      <c r="F59" s="3" t="inlineStr"/>
+      <c r="F59" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>rolling monthly broadband no contract</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr"/>
+          <t>broadband deals with no setup fee</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-deals-with-no-setup-fee (Caused by NameResolutionError("HTTPSConnection(host='broadbandpic</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>/guides/full-fibre-broadband-explained</t>
+          <t>/guides/best-rolling-monthly-broadband-deals</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -10382,18 +10730,24 @@
       </c>
       <c r="D60" s="2" t="inlineStr"/>
       <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>full fibre broadband explained</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr"/>
+          <t>rolling monthly broadband no contract</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-rolling-monthly-broadband-deals (Caused by NameResolutionError("HTTPSConnection(host='broadband</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>/guides/broadband-speeds-explained</t>
+          <t>/guides/full-fibre-broadband-explained</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -10408,18 +10762,24 @@
       </c>
       <c r="D61" s="3" t="inlineStr"/>
       <c r="E61" s="3" t="inlineStr"/>
-      <c r="F61" s="3" t="inlineStr"/>
+      <c r="F61" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>broadband speeds explained</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr"/>
+          <t>full fibre broadband explained</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/full-fibre-broadband-explained (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>/guides/cheapest-broadband-uk</t>
+          <t>/guides/broadband-speeds-explained</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -10434,18 +10794,24 @@
       </c>
       <c r="D62" s="2" t="inlineStr"/>
       <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>cheapest broadband uk, cheapest broadband deals uk</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr"/>
+          <t>broadband speeds explained</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-speeds-explained (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>/guides/best-broadband-for-working-from-home</t>
+          <t>/guides/cheapest-broadband-uk</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -10460,18 +10826,24 @@
       </c>
       <c r="D63" s="3" t="inlineStr"/>
       <c r="E63" s="3" t="inlineStr"/>
-      <c r="F63" s="3" t="inlineStr"/>
+      <c r="F63" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>best broadband for working from home</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr"/>
+          <t>cheapest broadband uk, cheapest broadband deals uk</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/cheapest-broadband-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk', </t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>/guides/best-broadband-for-students</t>
+          <t>/guides/best-broadband-for-working-from-home</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -10486,18 +10858,24 @@
       </c>
       <c r="D64" s="2" t="inlineStr"/>
       <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>best broadband for students</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr"/>
+          <t>best broadband for working from home</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-broadband-for-working-from-home (Caused by NameResolutionError("HTTPSConnection(host='broadband</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>/guides/best-broadband-for-streaming</t>
+          <t>/guides/best-broadband-for-students</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -10512,18 +10890,24 @@
       </c>
       <c r="D65" s="3" t="inlineStr"/>
       <c r="E65" s="3" t="inlineStr"/>
-      <c r="F65" s="3" t="inlineStr"/>
+      <c r="F65" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>best broadband for streaming</t>
-        </is>
-      </c>
-      <c r="H65" s="3" t="inlineStr"/>
+          <t>best broadband for students</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-broadband-for-students (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>/guides/best-broadband-providers-uk</t>
+          <t>/guides/best-broadband-for-streaming</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -10538,18 +10922,24 @@
       </c>
       <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr"/>
-      <c r="F66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>best broadband providers uk</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr"/>
+          <t>best broadband for streaming</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-broadband-for-streaming (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.c</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>/guides/broadband-price-rises-2026</t>
+          <t>/guides/best-broadband-providers-uk</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -10564,18 +10954,24 @@
       </c>
       <c r="D67" s="3" t="inlineStr"/>
       <c r="E67" s="3" t="inlineStr"/>
-      <c r="F67" s="3" t="inlineStr"/>
+      <c r="F67" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>broadband price rises 2026</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr"/>
+          <t>best broadband providers uk</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-broadband-providers-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>/guides/can-i-leave-broadband-early-after-price-rise</t>
+          <t>/guides/broadband-price-rises-2026</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -10590,18 +10986,24 @@
       </c>
       <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr"/>
-      <c r="F68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>can i leave broadband contract early</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr"/>
+          <t>broadband price rises 2026</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-price-rises-2026 (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>/guides/broadband-without-phone-line</t>
+          <t>/guides/can-i-leave-broadband-early-after-price-rise</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -10616,18 +11018,24 @@
       </c>
       <c r="D69" s="3" t="inlineStr"/>
       <c r="E69" s="3" t="inlineStr"/>
-      <c r="F69" s="3" t="inlineStr"/>
+      <c r="F69" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>broadband without landline, broadband without phone line</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr"/>
+          <t>can i leave broadband contract early</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/can-i-leave-broadband-early-after-price-rise (Caused by NameResolutionError("HTTPSConnection(host='b</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>/guides/best-5g-home-broadband-uk</t>
+          <t>/guides/broadband-without-phone-line</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -10642,18 +11050,24 @@
       </c>
       <c r="D70" s="2" t="inlineStr"/>
       <c r="E70" s="2" t="inlineStr"/>
-      <c r="F70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>best 5g home broadband uk</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr"/>
+          <t>broadband without landline, broadband without phone line</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-without-phone-line (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.c</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>/guides/best-full-fibre-broadband-uk</t>
+          <t>/guides/best-5g-home-broadband-uk</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -10668,18 +11082,24 @@
       </c>
       <c r="D71" s="3" t="inlineStr"/>
       <c r="E71" s="3" t="inlineStr"/>
-      <c r="F71" s="3" t="inlineStr"/>
+      <c r="F71" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>best full fibre broadband uk</t>
-        </is>
-      </c>
-      <c r="H71" s="3" t="inlineStr"/>
+          <t>best 5g home broadband uk</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-5g-home-broadband-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.u</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>/guides/best-broadband-for-gaming-uk</t>
+          <t>/guides/best-full-fibre-broadband-uk</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -10694,18 +11114,24 @@
       </c>
       <c r="D72" s="2" t="inlineStr"/>
       <c r="E72" s="2" t="inlineStr"/>
-      <c r="F72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>best broadband for gaming uk</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr"/>
+          <t>best full fibre broadband uk</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-full-fibre-broadband-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.c</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>/guides/broadband-social-tariffs-uk</t>
+          <t>/guides/best-broadband-for-gaming-uk</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -10720,18 +11146,24 @@
       </c>
       <c r="D73" s="3" t="inlineStr"/>
       <c r="E73" s="3" t="inlineStr"/>
-      <c r="F73" s="3" t="inlineStr"/>
+      <c r="F73" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>broadband social tariffs uk</t>
-        </is>
-      </c>
-      <c r="H73" s="3" t="inlineStr"/>
+          <t>best broadband for gaming uk</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-broadband-for-gaming-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.c</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>/guides/broadband-moving-house</t>
+          <t>/guides/broadband-social-tariffs-uk</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -10746,18 +11178,24 @@
       </c>
       <c r="D74" s="2" t="inlineStr"/>
       <c r="E74" s="2" t="inlineStr"/>
-      <c r="F74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>broadband when moving house</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr"/>
+          <t>broadband social tariffs uk</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-social-tariffs-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>/guides/best-broadband-for-rural-areas-uk</t>
+          <t>/guides/broadband-moving-house</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -10772,18 +11210,24 @@
       </c>
       <c r="D75" s="3" t="inlineStr"/>
       <c r="E75" s="3" t="inlineStr"/>
-      <c r="F75" s="3" t="inlineStr"/>
+      <c r="F75" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>best broadband for rural areas uk</t>
-        </is>
-      </c>
-      <c r="H75" s="3" t="inlineStr"/>
+          <t>broadband when moving house</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-moving-house (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.co.uk',</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>/guides/broadband-for-existing-customers</t>
+          <t>/guides/best-broadband-for-rural-areas-uk</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -10798,18 +11242,24 @@
       </c>
       <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr"/>
-      <c r="F76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>staying with existing broadband provider deals</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr"/>
+          <t>best broadband for rural areas uk</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/best-broadband-for-rural-areas-uk (Caused by NameResolutionError("HTTPSConnection(host='broadbandpic</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>/guides/one-touch-switching-explained</t>
+          <t>/guides/broadband-for-existing-customers</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -10824,18 +11274,24 @@
       </c>
       <c r="D77" s="3" t="inlineStr"/>
       <c r="E77" s="3" t="inlineStr"/>
-      <c r="F77" s="3" t="inlineStr"/>
+      <c r="F77" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>one touch switching broadband explained</t>
-        </is>
-      </c>
-      <c r="H77" s="3" t="inlineStr"/>
+          <t>staying with existing broadband provider deals</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-for-existing-customers (Caused by NameResolutionError("HTTPSConnection(host='broadbandpick</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>/guides/broadband-contract-end-rights</t>
+          <t>/guides/one-touch-switching-explained</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -10850,16 +11306,54 @@
       </c>
       <c r="D78" s="2" t="inlineStr"/>
       <c r="E78" s="2" t="inlineStr"/>
-      <c r="F78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
+          <t>one touch switching broadband explained</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/one-touch-switching-explained (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>/guides/broadband-contract-end-rights</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Editorial guide</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr"/>
+      <c r="E79" s="3" t="inlineStr"/>
+      <c r="F79" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
           <t>broadband contract end rights</t>
         </is>
       </c>
-      <c r="H78" s="2" t="inlineStr"/>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='broadbandpicker.co.uk', port=443): Max retries exceeded with url: /guides/broadband-contract-end-rights (Caused by NameResolutionError("HTTPSConnection(host='broadbandpicker.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H78"/>
+  <autoFilter ref="A1:H79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -13037,10 +13531,10 @@
         <v>29670</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>39.4</v>

</xml_diff>

<commit_message>
feat: persistent postcode across the site
- Add lib/postcodeStorage.ts: localStorage helper (get/set/clear) for the
  checked postcode, SSR-safe (guards typeof window)
- PostcodeChecker now persists the postcode on submit, in addition to
  navigating to /postcode/[area]
- Add components/PostcodeContextBar.tsx: a slim "Showing results for X"
  strip with change/clear actions, shown on /deals, /compare and
  /providers/[slug] when a postcode is stored. Renders null server-side
  (no hydration mismatch) and only appears once a postcode is actually set

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/broadbandpicker-keyword-mapping.xlsx
+++ b/docs/broadbandpicker-keyword-mapping.xlsx
@@ -94,10 +94,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9007,7 +9007,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>7722</v>
+        <v>11360</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -9111,7 +9111,7 @@
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>9904</v>
+        <v>10163</v>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
@@ -9168,9 +9168,19 @@
           <t>Page</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Broadband Cost Calculator | True Monthly Cost UK | BroadbandPicker</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Broadband cost calculator</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>5349</v>
+      </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>broadband cost per mbps calculator</t>
@@ -9501,7 +9511,7 @@
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>5365</v>
+        <v>5489</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
@@ -9537,7 +9547,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>5237</v>
+        <v>5361</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -9573,7 +9583,7 @@
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>5354</v>
+        <v>5484</v>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
@@ -9609,7 +9619,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>5342</v>
+        <v>5466</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -9645,7 +9655,7 @@
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>5224</v>
+        <v>5348</v>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
@@ -9681,7 +9691,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>5092</v>
+        <v>5218</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -9717,7 +9727,7 @@
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>5315</v>
+        <v>5439</v>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
@@ -9753,7 +9763,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>5184</v>
+        <v>5314</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
@@ -9789,7 +9799,7 @@
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>5083</v>
+        <v>5205</v>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
@@ -9825,7 +9835,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>5187</v>
+        <v>5311</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
@@ -9861,7 +9871,7 @@
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>5322</v>
+        <v>5452</v>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
@@ -9897,7 +9907,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>4994</v>
+        <v>5118</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -9933,7 +9943,7 @@
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>5177</v>
+        <v>5301</v>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
@@ -12541,7 +12551,7 @@
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>7722</v>
+        <v>9059</v>
       </c>
       <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr"/>
@@ -12573,7 +12583,7 @@
         </is>
       </c>
       <c r="F105" s="3" t="n">
-        <v>7761</v>
+        <v>9100</v>
       </c>
       <c r="G105" s="3" t="inlineStr"/>
       <c r="H105" s="3" t="inlineStr"/>
@@ -12605,7 +12615,7 @@
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>7391</v>
+        <v>8600</v>
       </c>
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr"/>
@@ -12637,7 +12647,7 @@
         </is>
       </c>
       <c r="F107" s="3" t="n">
-        <v>7722</v>
+        <v>9059</v>
       </c>
       <c r="G107" s="3" t="inlineStr"/>
       <c r="H107" s="3" t="inlineStr"/>
@@ -12669,7 +12679,7 @@
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>7722</v>
+        <v>9059</v>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr"/>
@@ -12701,7 +12711,7 @@
         </is>
       </c>
       <c r="F109" s="3" t="n">
-        <v>7395</v>
+        <v>8604</v>
       </c>
       <c r="G109" s="3" t="inlineStr"/>
       <c r="H109" s="3" t="inlineStr"/>
@@ -12733,7 +12743,7 @@
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>7750</v>
+        <v>9093</v>
       </c>
       <c r="G110" s="2" t="inlineStr"/>
       <c r="H110" s="2" t="inlineStr"/>
@@ -12765,7 +12775,7 @@
         </is>
       </c>
       <c r="F111" s="3" t="n">
-        <v>7750</v>
+        <v>9093</v>
       </c>
       <c r="G111" s="3" t="inlineStr"/>
       <c r="H111" s="3" t="inlineStr"/>
@@ -12797,7 +12807,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>7392</v>
+        <v>8603</v>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr"/>
@@ -12829,7 +12839,7 @@
         </is>
       </c>
       <c r="F113" s="3" t="n">
-        <v>7391</v>
+        <v>8600</v>
       </c>
       <c r="G113" s="3" t="inlineStr"/>
       <c r="H113" s="3" t="inlineStr"/>
@@ -12861,7 +12871,7 @@
         </is>
       </c>
       <c r="F114" s="2" t="n">
-        <v>7139</v>
+        <v>8216</v>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
@@ -12893,7 +12903,7 @@
         </is>
       </c>
       <c r="F115" s="3" t="n">
-        <v>7098</v>
+        <v>8175</v>
       </c>
       <c r="G115" s="3" t="inlineStr"/>
       <c r="H115" s="3" t="inlineStr"/>
@@ -12925,7 +12935,7 @@
         </is>
       </c>
       <c r="F116" s="2" t="n">
-        <v>7059</v>
+        <v>8134</v>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
       <c r="H116" s="2" t="inlineStr"/>
@@ -12957,7 +12967,7 @@
         </is>
       </c>
       <c r="F117" s="3" t="n">
-        <v>7494</v>
+        <v>8705</v>
       </c>
       <c r="G117" s="3" t="inlineStr"/>
       <c r="H117" s="3" t="inlineStr"/>
@@ -12989,7 +12999,7 @@
         </is>
       </c>
       <c r="F118" s="2" t="n">
-        <v>7059</v>
+        <v>8134</v>
       </c>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr"/>
@@ -13021,7 +13031,7 @@
         </is>
       </c>
       <c r="F119" s="3" t="n">
-        <v>7133</v>
+        <v>8212</v>
       </c>
       <c r="G119" s="3" t="inlineStr"/>
       <c r="H119" s="3" t="inlineStr"/>
@@ -13053,7 +13063,7 @@
         </is>
       </c>
       <c r="F120" s="2" t="n">
-        <v>7053</v>
+        <v>8130</v>
       </c>
       <c r="G120" s="2" t="inlineStr"/>
       <c r="H120" s="2" t="inlineStr"/>
@@ -13085,7 +13095,7 @@
         </is>
       </c>
       <c r="F121" s="3" t="n">
-        <v>7139</v>
+        <v>8216</v>
       </c>
       <c r="G121" s="3" t="inlineStr"/>
       <c r="H121" s="3" t="inlineStr"/>
@@ -13117,7 +13127,7 @@
         </is>
       </c>
       <c r="F122" s="2" t="n">
-        <v>6698</v>
+        <v>7641</v>
       </c>
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr"/>
@@ -13149,7 +13159,7 @@
         </is>
       </c>
       <c r="F123" s="3" t="n">
-        <v>7135</v>
+        <v>8212</v>
       </c>
       <c r="G123" s="3" t="inlineStr"/>
       <c r="H123" s="3" t="inlineStr"/>
@@ -13181,7 +13191,7 @@
         </is>
       </c>
       <c r="F124" s="2" t="n">
-        <v>7494</v>
+        <v>8705</v>
       </c>
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr"/>
@@ -13213,7 +13223,7 @@
         </is>
       </c>
       <c r="F125" s="3" t="n">
-        <v>7059</v>
+        <v>8134</v>
       </c>
       <c r="G125" s="3" t="inlineStr"/>
       <c r="H125" s="3" t="inlineStr"/>
@@ -13245,7 +13255,7 @@
         </is>
       </c>
       <c r="F126" s="2" t="n">
-        <v>7490</v>
+        <v>8701</v>
       </c>
       <c r="G126" s="2" t="inlineStr"/>
       <c r="H126" s="2" t="inlineStr"/>
@@ -13277,7 +13287,7 @@
         </is>
       </c>
       <c r="F127" s="3" t="n">
-        <v>7135</v>
+        <v>8212</v>
       </c>
       <c r="G127" s="3" t="inlineStr"/>
       <c r="H127" s="3" t="inlineStr"/>
@@ -13309,7 +13319,7 @@
         </is>
       </c>
       <c r="F128" s="2" t="n">
-        <v>7135</v>
+        <v>8212</v>
       </c>
       <c r="G128" s="2" t="inlineStr"/>
       <c r="H128" s="2" t="inlineStr"/>
@@ -13341,7 +13351,7 @@
         </is>
       </c>
       <c r="F129" s="3" t="n">
-        <v>6778</v>
+        <v>7723</v>
       </c>
       <c r="G129" s="3" t="inlineStr"/>
       <c r="H129" s="3" t="inlineStr"/>
@@ -13373,7 +13383,7 @@
         </is>
       </c>
       <c r="F130" s="2" t="n">
-        <v>7494</v>
+        <v>8705</v>
       </c>
       <c r="G130" s="2" t="inlineStr"/>
       <c r="H130" s="2" t="inlineStr"/>
@@ -13405,7 +13415,7 @@
         </is>
       </c>
       <c r="F131" s="3" t="n">
-        <v>7490</v>
+        <v>8701</v>
       </c>
       <c r="G131" s="3" t="inlineStr"/>
       <c r="H131" s="3" t="inlineStr"/>
@@ -13437,7 +13447,7 @@
         </is>
       </c>
       <c r="F132" s="2" t="n">
-        <v>7139</v>
+        <v>8216</v>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
       <c r="H132" s="2" t="inlineStr"/>
@@ -13469,7 +13479,7 @@
         </is>
       </c>
       <c r="F133" s="3" t="n">
-        <v>7139</v>
+        <v>8216</v>
       </c>
       <c r="G133" s="3" t="inlineStr"/>
       <c r="H133" s="3" t="inlineStr"/>
@@ -13501,7 +13511,7 @@
         </is>
       </c>
       <c r="F134" s="2" t="n">
-        <v>7139</v>
+        <v>8216</v>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
       <c r="H134" s="2" t="inlineStr"/>
@@ -13533,7 +13543,7 @@
         </is>
       </c>
       <c r="F135" s="3" t="n">
-        <v>7139</v>
+        <v>8216</v>
       </c>
       <c r="G135" s="3" t="inlineStr"/>
       <c r="H135" s="3" t="inlineStr"/>
@@ -13565,7 +13575,7 @@
         </is>
       </c>
       <c r="F136" s="2" t="n">
-        <v>7465</v>
+        <v>8670</v>
       </c>
       <c r="G136" s="2" t="inlineStr"/>
       <c r="H136" s="2" t="inlineStr"/>
@@ -13597,7 +13607,7 @@
         </is>
       </c>
       <c r="F137" s="3" t="n">
-        <v>7139</v>
+        <v>8216</v>
       </c>
       <c r="G137" s="3" t="inlineStr"/>
       <c r="H137" s="3" t="inlineStr"/>
@@ -13629,7 +13639,7 @@
         </is>
       </c>
       <c r="F138" s="2" t="n">
-        <v>7494</v>
+        <v>8705</v>
       </c>
       <c r="G138" s="2" t="inlineStr"/>
       <c r="H138" s="2" t="inlineStr"/>
@@ -13661,7 +13671,7 @@
         </is>
       </c>
       <c r="F139" s="3" t="n">
-        <v>6698</v>
+        <v>7641</v>
       </c>
       <c r="G139" s="3" t="inlineStr"/>
       <c r="H139" s="3" t="inlineStr"/>
@@ -13693,7 +13703,7 @@
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>7474</v>
+        <v>8685</v>
       </c>
       <c r="G140" s="2" t="inlineStr"/>
       <c r="H140" s="2" t="inlineStr"/>
@@ -13725,7 +13735,7 @@
         </is>
       </c>
       <c r="F141" s="3" t="n">
-        <v>7394</v>
+        <v>8603</v>
       </c>
       <c r="G141" s="3" t="inlineStr"/>
       <c r="H141" s="3" t="inlineStr"/>
@@ -13757,7 +13767,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>7053</v>
+        <v>8130</v>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
       <c r="H142" s="2" t="inlineStr"/>
@@ -13789,7 +13799,7 @@
         </is>
       </c>
       <c r="F143" s="3" t="n">
-        <v>7055</v>
+        <v>8130</v>
       </c>
       <c r="G143" s="3" t="inlineStr"/>
       <c r="H143" s="3" t="inlineStr"/>
@@ -13821,7 +13831,7 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>7053</v>
+        <v>8130</v>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
       <c r="H144" s="2" t="inlineStr"/>
@@ -13853,7 +13863,7 @@
         </is>
       </c>
       <c r="F145" s="3" t="n">
-        <v>7053</v>
+        <v>8130</v>
       </c>
       <c r="G145" s="3" t="inlineStr"/>
       <c r="H145" s="3" t="inlineStr"/>
@@ -13885,7 +13895,7 @@
         </is>
       </c>
       <c r="F146" s="2" t="n">
-        <v>7059</v>
+        <v>8134</v>
       </c>
       <c r="G146" s="2" t="inlineStr"/>
       <c r="H146" s="2" t="inlineStr"/>
@@ -13917,7 +13927,7 @@
         </is>
       </c>
       <c r="F147" s="3" t="n">
-        <v>6698</v>
+        <v>7641</v>
       </c>
       <c r="G147" s="3" t="inlineStr"/>
       <c r="H147" s="3" t="inlineStr"/>
@@ -13949,7 +13959,7 @@
         </is>
       </c>
       <c r="F148" s="2" t="n">
-        <v>7057</v>
+        <v>8134</v>
       </c>
       <c r="G148" s="2" t="inlineStr"/>
       <c r="H148" s="2" t="inlineStr"/>
@@ -13981,7 +13991,7 @@
         </is>
       </c>
       <c r="F149" s="3" t="n">
-        <v>7494</v>
+        <v>8705</v>
       </c>
       <c r="G149" s="3" t="inlineStr"/>
       <c r="H149" s="3" t="inlineStr"/>
@@ -14013,7 +14023,7 @@
         </is>
       </c>
       <c r="F150" s="2" t="n">
-        <v>7059</v>
+        <v>8134</v>
       </c>
       <c r="G150" s="2" t="inlineStr"/>
       <c r="H150" s="2" t="inlineStr"/>
@@ -14045,7 +14055,7 @@
         </is>
       </c>
       <c r="F151" s="3" t="n">
-        <v>7098</v>
+        <v>8175</v>
       </c>
       <c r="G151" s="3" t="inlineStr"/>
       <c r="H151" s="3" t="inlineStr"/>
@@ -14077,7 +14087,7 @@
         </is>
       </c>
       <c r="F152" s="2" t="n">
-        <v>7053</v>
+        <v>8130</v>
       </c>
       <c r="G152" s="2" t="inlineStr"/>
       <c r="H152" s="2" t="inlineStr"/>
@@ -14109,7 +14119,7 @@
         </is>
       </c>
       <c r="F153" s="3" t="n">
-        <v>7055</v>
+        <v>8130</v>
       </c>
       <c r="G153" s="3" t="inlineStr"/>
       <c r="H153" s="3" t="inlineStr"/>
@@ -14236,34 +14246,34 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/tools/broadband-cost-calculator</t>
+          <t>https://broadbandpicker.co.uk/providers/onestream</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Broadband cost calculator: true monthly and contract-length cost</t>
+          <t>Onestream — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Tools</t>
+          <t>Provider brand</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Interactive tool</t>
+          <t>Provider page</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>broadband cost per mbps calculator</t>
+          <t>onestream broadband</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>210</v>
+        <v>880</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -14271,14 +14281,14 @@
         </is>
       </c>
       <c r="L2" s="2" t="n">
-        <v>59.9</v>
+        <v>59.4</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>27.6</v>
+        <v>28</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Very easy opportunity (difficulty 16); niche combined demand (210/mo); supporting intent; covers 1 mapped keyword.</t>
+          <t>Very easy opportunity (difficulty 18); useful combined demand (880/mo); supporting intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14298,49 +14308,49 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/onestream</t>
+          <t>https://broadbandpicker.co.uk/guides/no-credit-check-broadband-uk</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Onestream — plans, coverage and Awin-tracked deals</t>
+          <t>No credit check broadband in the UK: options and what to expect</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Provider brand</t>
+          <t>Affordability</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Provider page</t>
+          <t>Guide</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>onestream broadband</t>
+          <t>no credit check broadband</t>
         </is>
       </c>
       <c r="I3" s="3" t="n">
-        <v>880</v>
+        <v>1900</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="L3" s="3" t="n">
-        <v>59.4</v>
+        <v>59.3</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>28</v>
+        <v>34.8</v>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>Very easy opportunity (difficulty 18); useful combined demand (880/mo); supporting intent; covers 1 mapped keyword.</t>
+          <t>Moderate opportunity (difficulty 32); strong combined demand (1,900/mo); commercial intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14360,49 +14370,49 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/guides/no-credit-check-broadband-uk</t>
+          <t>https://broadbandpicker.co.uk/providers/brsk</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>No credit check broadband in the UK: options and what to expect</t>
+          <t>Brsk — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Affordability</t>
+          <t>Provider brand</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Guide</t>
+          <t>Provider page</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>no credit check broadband</t>
+          <t>brsk broadband</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
         <v>1900</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Very easy</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
-        <v>59.3</v>
+        <v>59</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>34.8</v>
+        <v>28.5</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Moderate opportunity (difficulty 32); strong combined demand (1,900/mo); commercial intent; covers 1 mapped keyword.</t>
+          <t>Very easy opportunity (difficulty 20); strong combined demand (1,900/mo); supporting intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14422,31 +14432,31 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/brsk</t>
+          <t>https://broadbandpicker.co.uk/guides/fttp-vs-fttc-explained</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Brsk — plans, coverage and Awin-tracked deals</t>
+          <t>FTTP vs FTTC: what the difference means for your speed</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Provider brand</t>
+          <t>Technology &amp; speeds</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Provider page</t>
+          <t>Guide</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>brsk broadband</t>
+          <t>fttp vs fttc explained</t>
         </is>
       </c>
       <c r="I5" s="3" t="n">
-        <v>1900</v>
+        <v>880</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>20</v>
@@ -14457,14 +14467,14 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>59</v>
+        <v>58.4</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>28.5</v>
+        <v>27.8</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>Very easy opportunity (difficulty 20); strong combined demand (1,900/mo); supporting intent; covers 1 mapped keyword.</t>
+          <t>Very easy opportunity (difficulty 20); useful combined demand (880/mo); supporting intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14484,12 +14494,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/guides/fttp-vs-fttc-explained</t>
+          <t>https://broadbandpicker.co.uk/guides/best-mesh-wifi-for-your-broadband-router</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>FTTP vs FTTC: what the difference means for your speed</t>
+          <t>Best mesh Wi-Fi systems to pair with your broadband router</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -14504,29 +14514,29 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>fttp vs fttc explained</t>
+          <t>best mesh wifi for broadband router</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>880</v>
+        <v>1300</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
         <v>58.4</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>27.8</v>
+        <v>34</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Very easy opportunity (difficulty 20); useful combined demand (880/mo); supporting intent; covers 1 mapped keyword.</t>
+          <t>Moderate opportunity (difficulty 33); strong combined demand (1,300/mo); commercial intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14546,17 +14556,17 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/guides/best-mesh-wifi-for-your-broadband-router</t>
+          <t>https://broadbandpicker.co.uk/guides/broadband-help-if-you-claim-benefits-uk</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Best mesh Wi-Fi systems to pair with your broadband router</t>
+          <t>Cheaper broadband if you claim benefits: social tariffs explained</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Technology &amp; speeds</t>
+          <t>Affordability</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -14566,29 +14576,29 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>best mesh wifi for broadband router</t>
+          <t>broadband for universal credit</t>
         </is>
       </c>
       <c r="I7" s="3" t="n">
-        <v>1300</v>
+        <v>720</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Very easy</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>58.4</v>
+        <v>58.2</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>34</v>
+        <v>27.5</v>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>Moderate opportunity (difficulty 33); strong combined demand (1,300/mo); commercial intent; covers 1 mapped keyword.</t>
+          <t>Very easy opportunity (difficulty 20); useful combined demand (720/mo); supporting intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14608,49 +14618,49 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/guides/broadband-help-if-you-claim-benefits-uk</t>
+          <t>https://broadbandpicker.co.uk/providers/gigaclear</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Cheaper broadband if you claim benefits: social tariffs explained</t>
+          <t>Gigaclear — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Affordability</t>
+          <t>Provider brand</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Guide</t>
+          <t>Provider page</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>broadband for universal credit</t>
+          <t>gigaclear broadband</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>720</v>
+        <v>2400</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Very easy</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="L8" s="2" t="n">
-        <v>58.2</v>
+        <v>56.9</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>27.5</v>
+        <v>27.9</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Very easy opportunity (difficulty 20); useful combined demand (720/mo); supporting intent; covers 1 mapped keyword.</t>
+          <t>Easy opportunity (difficulty 24); strong combined demand (2,400/mo); supporting intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14670,12 +14680,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/gigaclear</t>
+          <t>https://broadbandpicker.co.uk/providers/cuckoo</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Gigaclear — plans, coverage and Awin-tracked deals</t>
+          <t>Cuckoo Broadband — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -14690,14 +14700,14 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>gigaclear broadband</t>
+          <t>cuckoo broadband broadband</t>
         </is>
       </c>
       <c r="I9" s="3" t="n">
-        <v>2400</v>
+        <v>2900</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -14705,14 +14715,14 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>56.9</v>
+        <v>56.5</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>27.9</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>Easy opportunity (difficulty 24); strong combined demand (2,400/mo); supporting intent; covers 1 mapped keyword.</t>
+          <t>Easy opportunity (difficulty 25); strong combined demand (2,900/mo); supporting intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14732,49 +14742,49 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/cuckoo</t>
+          <t>https://broadbandpicker.co.uk/guides/black-friday-broadband-deals-uk</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Cuckoo Broadband — plans, coverage and Awin-tracked deals</t>
+          <t>Black Friday broadband deals UK: what to expect and how to compare</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Provider brand</t>
+          <t>Deals &amp; pricing</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Provider page</t>
+          <t>Guide</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>cuckoo broadband broadband</t>
+          <t>black friday broadband deals</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>2900</v>
+        <v>5400</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Competitive</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
-        <v>56.5</v>
+        <v>55.8</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>27.9</v>
+        <v>37</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Easy opportunity (difficulty 25); strong combined demand (2,900/mo); supporting intent; covers 1 mapped keyword.</t>
+          <t>Competitive opportunity (difficulty 42); strong combined demand (5,400/mo); commercial intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14794,49 +14804,49 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/guides/black-friday-broadband-deals-uk</t>
+          <t>https://broadbandpicker.co.uk/providers/shell-energy</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Black Friday broadband deals UK: what to expect and how to compare</t>
+          <t>Shell Energy Broadband — plans, coverage and Awin-tracked deals</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Deals &amp; pricing</t>
+          <t>Provider brand</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Guide</t>
+          <t>Provider page</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>black friday broadband deals</t>
+          <t>shell energy broadband broadband</t>
         </is>
       </c>
       <c r="I11" s="3" t="n">
-        <v>5400</v>
+        <v>3600</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Competitive</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>55.8</v>
+        <v>55.7</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>Competitive opportunity (difficulty 42); strong combined demand (5,400/mo); commercial intent; covers 1 mapped keyword.</t>
+          <t>Easy opportunity (difficulty 27); strong combined demand (3,600/mo); supporting intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14856,31 +14866,31 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/providers/shell-energy</t>
+          <t>https://broadbandpicker.co.uk/research/broadband-customer-service-rankings-uk</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Shell Energy Broadband — plans, coverage and Awin-tracked deals</t>
+          <t>Broadband customer service rankings: Ofcom-evidenced comparison</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Provider brand</t>
+          <t>Trust &amp; research</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Provider page</t>
+          <t>Research page</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>shell energy broadband broadband</t>
+          <t>best customer service broadband provider</t>
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>3600</v>
+        <v>880</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>27</v>
@@ -14891,14 +14901,14 @@
         </is>
       </c>
       <c r="L12" s="2" t="n">
-        <v>55.7</v>
+        <v>55.1</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>28</v>
+        <v>27.8</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Easy opportunity (difficulty 27); strong combined demand (3,600/mo); supporting intent; covers 1 mapped keyword.</t>
+          <t>Easy opportunity (difficulty 27); useful combined demand (880/mo); supporting intent; covers 1 mapped keyword.</t>
         </is>
       </c>
     </row>
@@ -14918,12 +14928,12 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>https://broadbandpicker.co.uk/research/broadband-customer-service-rankings-uk</t>
+          <t>https://broadbandpicker.co.uk/guides/broadband-complaints-and-ombudsman-uk</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Broadband customer service rankings: Ofcom-evidenced comparison</t>
+          <t>Broadband complaints and the ombudsman: your UK rights</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -14933,1294 +14943,1292 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Research page</t>
+          <t>Guide</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>best customer service broadband provider</t>
+          <t>broadband complaints ombudsman</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
+        <v>720</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 26); useful combined demand (720/mo); supporting intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/compare/hyperoptic-vs-youfibre</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Hyperoptic vs YouFibre broadband: which is better in 2026?</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Provider vs comparison</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Comparison page</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>hyperoptic vs youfibre broadband</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Very easy</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Very easy opportunity (difficulty 14); niche combined demand (140/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/postcode/sheffield</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Broadband providers in Sheffield: coverage and best deals</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Postcode &amp; location</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>City hub</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>broadband providers sheffield</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>590</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Very easy</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Very easy opportunity (difficulty 19); useful combined demand (590/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/guides/static-ip-business-broadband-explained</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Static IP business broadband: when you need one and how much it costs</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Business broadband</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>static ip business broadband</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>480</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 24); useful combined demand (480/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/guides/student-broadband-by-university-city</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Student broadband by university city: short-term and rolling deals</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Use cases &amp; lifestyle</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>student broadband cities guide</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>320</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Very easy</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Very easy opportunity (difficulty 18); useful combined demand (320/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/postcode/edinburgh</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Broadband providers in Edinburgh: coverage and best deals</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Postcode &amp; location</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>City hub</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>broadband providers edinburgh</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>720</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 21); useful combined demand (720/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/guides/small-office-broadband-setup-uk</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Small office broadband setup: routers, backup and support checklist</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Business broadband</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>small office broadband setup</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>390</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 22); useful combined demand (390/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/compare/bt-vs-plusnet</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>BT vs Plusnet broadband: which is better in 2026?</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Provider vs comparison</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Comparison page</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>bt vs plusnet broadband</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>320</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Very easy</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Very easy opportunity (difficulty 19); useful combined demand (320/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/postcode/glasgow</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Broadband providers in Glasgow: coverage and best deals</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Postcode &amp; location</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>City hub</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>broadband providers glasgow</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="n">
         <v>880</v>
       </c>
-      <c r="J13" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="J21" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="L13" s="3" t="n">
-        <v>55.1</v>
-      </c>
-      <c r="M13" s="3" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="N13" s="3" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 27); useful combined demand (880/mo); supporting intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Planned — not live</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="L21" s="5" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="M21" s="5" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 22); useful combined demand (880/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/broadband-complaints-and-ombudsman-uk</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Broadband complaints and the ombudsman: your UK rights</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Trust &amp; research</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/postcode/liverpool</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Broadband providers in Liverpool: coverage and best deals</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Postcode &amp; location</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>City hub</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>broadband providers liverpool</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>880</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 22); useful combined demand (880/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr"/>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/guides/broadband-for-landlords-and-hmos-uk</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Broadband for landlords and HMOs: what to set up and who pays</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Use cases &amp; lifestyle</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Guide</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>broadband complaints ombudsman</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="n">
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>broadband for landlords hmo</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>480</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Very easy</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="M23" s="5" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>Very easy opportunity (difficulty 20); useful combined demand (480/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/postcode/leeds</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Broadband providers in Leeds: coverage and best deals</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Postcode &amp; location</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>City hub</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>broadband providers leeds</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 23); strong combined demand (1,000/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/compare/ee-vs-talktalk</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>EE vs TalkTalk broadband: which is better in 2026?</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Provider vs comparison</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Comparison page</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>ee vs talktalk broadband</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>390</v>
+      </c>
+      <c r="J25" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Very easy</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="M25" s="5" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Very easy opportunity (difficulty 20); useful combined demand (390/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr"/>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/postcode/bristol</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Broadband providers in Bristol: coverage and best deals</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Postcode &amp; location</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>City hub</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>broadband providers bristol</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>1300</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 24); strong combined demand (1,300/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/postcode/birmingham</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Broadband providers in Birmingham: coverage and best deals</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Postcode &amp; location</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>City hub</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>broadband providers birmingham</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="M27" s="5" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 25); strong combined demand (1,600/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/postcode/manchester</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Broadband providers in Manchester: coverage and best deals</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Postcode &amp; location</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>City hub</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>broadband providers manchester</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>1900</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 26); strong combined demand (1,900/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/guides/leased-line-cost-uk-explained</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Leased line cost UK: what small businesses actually pay</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Business broadband</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>leased line cost uk</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="n">
         <v>720</v>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J29" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="M29" s="5" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 30); useful combined demand (720/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/guides/starlink-vs-fibre-broadband-uk</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Starlink vs fibre broadband: when satellite makes sense in the UK</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Alternative access</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>starlink vs openreach broadband</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>590</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 24); useful combined demand (590/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/compare/virgin-media-vs-sky</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Virgin Media vs Sky broadband: which is better in 2026?</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Provider vs comparison</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Comparison page</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>virgin media vs sky broadband</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>880</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="M31" s="5" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 25); useful combined demand (880/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr"/>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/guides/january-broadband-deals-uk</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>January broadband deals UK: new-year switching guide</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Deals &amp; pricing</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>january broadband deals</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>1300</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>Easy opportunity (difficulty 28); strong combined demand (1,300/mo); commercial intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/tools/broadband-cost-calculator</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Broadband cost calculator: true monthly and contract-length cost</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Tools</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Interactive tool</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>broadband cost per mbps calculator</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>210</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>Very easy</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="M33" s="5" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>Very easy opportunity (difficulty 16); niche combined demand (210/mo); supporting intent; covers 1 mapped keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Built, live and deployed on Vercel</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>https://broadbandpicker.co.uk/providers/youfibre</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>YouFibre — plans, coverage and Awin-tracked deals</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Provider brand</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Provider page</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>youfibre broadband</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>4400</v>
+      </c>
+      <c r="J34" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K34" s="4" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="L14" s="2" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 26); useful combined demand (720/mo); supporting intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/compare/hyperoptic-vs-youfibre</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Hyperoptic vs YouFibre broadband: which is better in 2026?</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Provider vs comparison</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Comparison page</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>hyperoptic vs youfibre broadband</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="n">
-        <v>140</v>
-      </c>
-      <c r="J15" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="n">
-        <v>67.90000000000001</v>
-      </c>
-      <c r="M15" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t>Very easy opportunity (difficulty 14); niche combined demand (140/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr"/>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/postcode/sheffield</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Broadband providers in Sheffield: coverage and best deals</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>Postcode &amp; location</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>City hub</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>broadband providers sheffield</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="n">
-        <v>590</v>
-      </c>
-      <c r="J16" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="n">
-        <v>66.8</v>
-      </c>
-      <c r="M16" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="N16" s="5" t="inlineStr">
-        <is>
-          <t>Very easy opportunity (difficulty 19); useful combined demand (590/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/static-ip-business-broadband-explained</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Static IP business broadband: when you need one and how much it costs</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Business broadband</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>static ip business broadband</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>480</v>
-      </c>
-      <c r="J17" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="n">
-        <v>66.3</v>
-      </c>
-      <c r="M17" s="4" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 24); useful combined demand (480/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/student-broadband-by-university-city</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Student broadband by university city: short-term and rolling deals</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>Use cases &amp; lifestyle</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>student broadband cities guide</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>320</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="L18" s="5" t="n">
-        <v>65.90000000000001</v>
-      </c>
-      <c r="M18" s="5" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="N18" s="5" t="inlineStr">
-        <is>
-          <t>Very easy opportunity (difficulty 18); useful combined demand (320/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr"/>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/postcode/edinburgh</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Broadband providers in Edinburgh: coverage and best deals</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Postcode &amp; location</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>City hub</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>broadband providers edinburgh</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>720</v>
-      </c>
-      <c r="J19" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="n">
-        <v>65.8</v>
-      </c>
-      <c r="M19" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 21); useful combined demand (720/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr"/>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/small-office-broadband-setup-uk</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Small office broadband setup: routers, backup and support checklist</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>Business broadband</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>small office broadband setup</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>390</v>
-      </c>
-      <c r="J20" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="K20" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L20" s="5" t="n">
-        <v>65.8</v>
-      </c>
-      <c r="M20" s="5" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="N20" s="5" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 22); useful combined demand (390/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/compare/bt-vs-plusnet</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>BT vs Plusnet broadband: which is better in 2026?</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Provider vs comparison</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Comparison page</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>bt vs plusnet broadband</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="n">
-        <v>320</v>
-      </c>
-      <c r="J21" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="M21" s="4" t="n">
-        <v>36.4</v>
-      </c>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t>Very easy opportunity (difficulty 19); useful combined demand (320/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr"/>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/postcode/glasgow</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Broadband providers in Glasgow: coverage and best deals</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Postcode &amp; location</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>City hub</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>broadband providers glasgow</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="n">
-        <v>880</v>
-      </c>
-      <c r="J22" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="K22" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L22" s="5" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="M22" s="5" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="N22" s="5" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 22); useful combined demand (880/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/postcode/liverpool</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Broadband providers in Liverpool: coverage and best deals</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Postcode &amp; location</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>City hub</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>broadband providers liverpool</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="n">
-        <v>880</v>
-      </c>
-      <c r="J23" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="M23" s="4" t="n">
-        <v>40.1</v>
-      </c>
-      <c r="N23" s="4" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 22); useful combined demand (880/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr"/>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/broadband-for-landlords-and-hmos-uk</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Broadband for landlords and HMOs: what to set up and who pays</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Use cases &amp; lifestyle</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>broadband for landlords hmo</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="n">
-        <v>480</v>
-      </c>
-      <c r="J24" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="L24" s="5" t="n">
-        <v>65.09999999999999</v>
-      </c>
-      <c r="M24" s="5" t="n">
-        <v>36.6</v>
-      </c>
-      <c r="N24" s="5" t="inlineStr">
-        <is>
-          <t>Very easy opportunity (difficulty 20); useful combined demand (480/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr"/>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/postcode/leeds</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Broadband providers in Leeds: coverage and best deals</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Postcode &amp; location</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>City hub</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>broadband providers leeds</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J25" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="n">
-        <v>65.09999999999999</v>
-      </c>
-      <c r="M25" s="4" t="n">
-        <v>40.3</v>
-      </c>
-      <c r="N25" s="4" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 23); strong combined demand (1,000/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/compare/ee-vs-talktalk</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>EE vs TalkTalk broadband: which is better in 2026?</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Provider vs comparison</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>Comparison page</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>ee vs talktalk broadband</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="n">
-        <v>390</v>
-      </c>
-      <c r="J26" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>Very easy</t>
-        </is>
-      </c>
-      <c r="L26" s="5" t="n">
-        <v>65</v>
-      </c>
-      <c r="M26" s="5" t="n">
-        <v>36.4</v>
-      </c>
-      <c r="N26" s="5" t="inlineStr">
-        <is>
-          <t>Very easy opportunity (difficulty 20); useful combined demand (390/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr"/>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/postcode/bristol</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>Broadband providers in Bristol: coverage and best deals</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Postcode &amp; location</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>City hub</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>broadband providers bristol</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="n">
-        <v>1300</v>
-      </c>
-      <c r="J27" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="n">
-        <v>64.90000000000001</v>
-      </c>
-      <c r="M27" s="4" t="n">
-        <v>40.8</v>
-      </c>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 24); strong combined demand (1,300/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr"/>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/postcode/birmingham</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Broadband providers in Birmingham: coverage and best deals</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Postcode &amp; location</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>City hub</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>broadband providers birmingham</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="n">
-        <v>1600</v>
-      </c>
-      <c r="J28" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="K28" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L28" s="5" t="n">
-        <v>64.5</v>
-      </c>
-      <c r="M28" s="5" t="n">
-        <v>41.1</v>
-      </c>
-      <c r="N28" s="5" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 25); strong combined demand (1,600/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr"/>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/postcode/manchester</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Broadband providers in Manchester: coverage and best deals</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Postcode &amp; location</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>City hub</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>broadband providers manchester</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="n">
-        <v>1900</v>
-      </c>
-      <c r="J29" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="n">
-        <v>64.2</v>
-      </c>
-      <c r="M29" s="4" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 26); strong combined demand (1,900/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr"/>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/leased-line-cost-uk-explained</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Leased line cost UK: what small businesses actually pay</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Business broadband</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>leased line cost uk</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="n">
-        <v>720</v>
-      </c>
-      <c r="J30" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="K30" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L30" s="5" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="M30" s="5" t="n">
-        <v>58.6</v>
-      </c>
-      <c r="N30" s="5" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 30); useful combined demand (720/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr"/>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/starlink-vs-fibre-broadband-uk</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Starlink vs fibre broadband: when satellite makes sense in the UK</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Alternative access</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>starlink vs openreach broadband</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="n">
-        <v>590</v>
-      </c>
-      <c r="J31" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="M31" s="4" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 24); useful combined demand (590/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr"/>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/compare/virgin-media-vs-sky</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Virgin Media vs Sky broadband: which is better in 2026?</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Provider vs comparison</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>Comparison page</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>virgin media vs sky broadband</t>
-        </is>
-      </c>
-      <c r="I32" s="5" t="n">
-        <v>880</v>
-      </c>
-      <c r="J32" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="K32" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L32" s="5" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="M32" s="5" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="N32" s="5" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 25); useful combined demand (880/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr"/>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/guides/january-broadband-deals-uk</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>January broadband deals UK: new-year switching guide</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Deals &amp; pricing</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>january broadband deals</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="n">
-        <v>1300</v>
-      </c>
-      <c r="J33" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="n">
-        <v>61.7</v>
-      </c>
-      <c r="M33" s="4" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="N33" s="4" t="inlineStr">
-        <is>
-          <t>Easy opportunity (difficulty 28); strong combined demand (1,300/mo); commercial intent; covers 1 mapped keyword.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Built, live and deployed on Vercel</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>https://broadbandpicker.co.uk/providers/youfibre</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>YouFibre — plans, coverage and Awin-tracked deals</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>Provider brand</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>Provider page</t>
-        </is>
-      </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>youfibre broadband</t>
-        </is>
-      </c>
-      <c r="I34" s="5" t="n">
-        <v>4400</v>
-      </c>
-      <c r="J34" s="5" t="n">
-        <v>26</v>
-      </c>
-      <c r="K34" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="L34" s="5" t="n">
+      <c r="L34" s="4" t="n">
         <v>56.6</v>
       </c>
-      <c r="M34" s="5" t="n">
+      <c r="M34" s="4" t="n">
         <v>28.7</v>
       </c>
-      <c r="N34" s="5" t="inlineStr">
+      <c r="N34" s="4" t="inlineStr">
         <is>
           <t>Easy opportunity (difficulty 26); strong combined demand (4,400/mo); supporting intent; covers 1 mapped keyword.</t>
         </is>

</xml_diff>

<commit_message>
docs: research and plan the Broadband Match recommendation quiz
- Add a Strategic Lens section to docs/page-build-pipeline-brief.md: check
  whether a proposed feature already exists among competitors before
  building it, differentiate rather than clone, weight genuine gaps higher
  in tracker priority, and pair any interactive-only tool with static
  citable content since AI Overviews cite pages, not live tool output
- Research (WebSearch/WebFetch across Uswitch, Compare the Market,
  MoneySuperMarket, Which?, broadbandchoices, choose.co.uk,
  broadband.co.uk, and the closest analog RightSpeed UK) confirms a
  personalised quiz that outputs a ranked provider/package recommendation
  is a genuine gap, not a crowded feature
- Add feat-broadband-match-quiz to scripts/build_master_tracker.py with a
  research-informed priority score (78) — now the top pending item

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/broadbandpicker-keyword-mapping.xlsx
+++ b/docs/broadbandpicker-keyword-mapping.xlsx
@@ -627,7 +627,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>None supplied</t>
+          <t>https://docs.google.com/spreadsheets/d/1_IeyaXe1fSbXmV8Z4MdVOigMIz-cgK2h/edit</t>
         </is>
       </c>
     </row>
@@ -9111,7 +9111,7 @@
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>10163</v>
+        <v>10416</v>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
@@ -11487,7 +11487,7 @@
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>9058</v>
+        <v>9062</v>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
@@ -13764,19 +13764,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>KT1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E142" s="2" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Kingston upon Thames ( KT1 )</t>
-        </is>
-      </c>
-      <c r="F142" s="2" t="n">
-        <v>8685</v>
-      </c>
+      <c r="D142" s="2" t="inlineStr"/>
+      <c r="E142" s="2" t="inlineStr"/>
+      <c r="F142" s="2" t="inlineStr"/>
       <c r="G142" s="2" t="inlineStr"/>
       <c r="H142" s="2" t="inlineStr"/>
     </row>
@@ -13796,19 +13786,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D143" s="3" t="inlineStr">
-        <is>
-          <t>CR0 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E143" s="3" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Croydon ( CR0 )</t>
-        </is>
-      </c>
-      <c r="F143" s="3" t="n">
-        <v>8603</v>
-      </c>
+      <c r="D143" s="3" t="inlineStr"/>
+      <c r="E143" s="3" t="inlineStr"/>
+      <c r="F143" s="3" t="inlineStr"/>
       <c r="G143" s="3" t="inlineStr"/>
       <c r="H143" s="3" t="inlineStr"/>
     </row>
@@ -13828,19 +13808,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t>HA1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E144" s="2" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Harrow ( HA1 )</t>
-        </is>
-      </c>
-      <c r="F144" s="2" t="n">
-        <v>8130</v>
-      </c>
+      <c r="D144" s="2" t="inlineStr"/>
+      <c r="E144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="inlineStr"/>
       <c r="G144" s="2" t="inlineStr"/>
       <c r="H144" s="2" t="inlineStr"/>
     </row>
@@ -13860,19 +13830,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D145" s="3" t="inlineStr">
-        <is>
-          <t>UB1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E145" s="3" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Southall ( UB1 )</t>
-        </is>
-      </c>
-      <c r="F145" s="3" t="n">
-        <v>8130</v>
-      </c>
+      <c r="D145" s="3" t="inlineStr"/>
+      <c r="E145" s="3" t="inlineStr"/>
+      <c r="F145" s="3" t="inlineStr"/>
       <c r="G145" s="3" t="inlineStr"/>
       <c r="H145" s="3" t="inlineStr"/>
     </row>
@@ -13892,19 +13852,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D146" s="2" t="inlineStr">
-        <is>
-          <t>EN1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E146" s="2" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Enfield ( EN1 )</t>
-        </is>
-      </c>
-      <c r="F146" s="2" t="n">
-        <v>8130</v>
-      </c>
+      <c r="D146" s="2" t="inlineStr"/>
+      <c r="E146" s="2" t="inlineStr"/>
+      <c r="F146" s="2" t="inlineStr"/>
       <c r="G146" s="2" t="inlineStr"/>
       <c r="H146" s="2" t="inlineStr"/>
     </row>
@@ -13924,19 +13874,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D147" s="3" t="inlineStr">
-        <is>
-          <t>RM1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E147" s="3" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Romford ( RM1 )</t>
-        </is>
-      </c>
-      <c r="F147" s="3" t="n">
-        <v>8130</v>
-      </c>
+      <c r="D147" s="3" t="inlineStr"/>
+      <c r="E147" s="3" t="inlineStr"/>
+      <c r="F147" s="3" t="inlineStr"/>
       <c r="G147" s="3" t="inlineStr"/>
       <c r="H147" s="3" t="inlineStr"/>
     </row>
@@ -13956,19 +13896,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D148" s="2" t="inlineStr">
-        <is>
-          <t>DA1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E148" s="2" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Dartford ( DA1 )</t>
-        </is>
-      </c>
-      <c r="F148" s="2" t="n">
-        <v>8134</v>
-      </c>
+      <c r="D148" s="2" t="inlineStr"/>
+      <c r="E148" s="2" t="inlineStr"/>
+      <c r="F148" s="2" t="inlineStr"/>
       <c r="G148" s="2" t="inlineStr"/>
       <c r="H148" s="2" t="inlineStr"/>
     </row>
@@ -13988,19 +13918,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D149" s="3" t="inlineStr">
-        <is>
-          <t>ME1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E149" s="3" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Rochester ( ME1 )</t>
-        </is>
-      </c>
-      <c r="F149" s="3" t="n">
-        <v>7641</v>
-      </c>
+      <c r="D149" s="3" t="inlineStr"/>
+      <c r="E149" s="3" t="inlineStr"/>
+      <c r="F149" s="3" t="inlineStr"/>
       <c r="G149" s="3" t="inlineStr"/>
       <c r="H149" s="3" t="inlineStr"/>
     </row>
@@ -14020,19 +13940,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D150" s="2" t="inlineStr">
-        <is>
-          <t>SL1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E150" s="2" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Slough ( SL1 )</t>
-        </is>
-      </c>
-      <c r="F150" s="2" t="n">
-        <v>8134</v>
-      </c>
+      <c r="D150" s="2" t="inlineStr"/>
+      <c r="E150" s="2" t="inlineStr"/>
+      <c r="F150" s="2" t="inlineStr"/>
       <c r="G150" s="2" t="inlineStr"/>
       <c r="H150" s="2" t="inlineStr"/>
     </row>
@@ -14052,19 +13962,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D151" s="3" t="inlineStr">
-        <is>
-          <t>RG1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E151" s="3" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Reading Town Centre ( RG1 )</t>
-        </is>
-      </c>
-      <c r="F151" s="3" t="n">
-        <v>8705</v>
-      </c>
+      <c r="D151" s="3" t="inlineStr"/>
+      <c r="E151" s="3" t="inlineStr"/>
+      <c r="F151" s="3" t="inlineStr"/>
       <c r="G151" s="3" t="inlineStr"/>
       <c r="H151" s="3" t="inlineStr"/>
     </row>
@@ -14084,19 +13984,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D152" s="2" t="inlineStr">
-        <is>
-          <t>GU1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E152" s="2" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Guildford ( GU1 )</t>
-        </is>
-      </c>
-      <c r="F152" s="2" t="n">
-        <v>8134</v>
-      </c>
+      <c r="D152" s="2" t="inlineStr"/>
+      <c r="E152" s="2" t="inlineStr"/>
+      <c r="F152" s="2" t="inlineStr"/>
       <c r="G152" s="2" t="inlineStr"/>
       <c r="H152" s="2" t="inlineStr"/>
     </row>
@@ -14116,19 +14006,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D153" s="3" t="inlineStr">
-        <is>
-          <t>MK1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E153" s="3" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Milton Keynes ( MK1 )</t>
-        </is>
-      </c>
-      <c r="F153" s="3" t="n">
-        <v>8175</v>
-      </c>
+      <c r="D153" s="3" t="inlineStr"/>
+      <c r="E153" s="3" t="inlineStr"/>
+      <c r="F153" s="3" t="inlineStr"/>
       <c r="G153" s="3" t="inlineStr"/>
       <c r="H153" s="3" t="inlineStr"/>
     </row>
@@ -14148,19 +14028,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D154" s="2" t="inlineStr">
-        <is>
-          <t>LU1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E154" s="2" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Luton ( LU1 )</t>
-        </is>
-      </c>
-      <c r="F154" s="2" t="n">
-        <v>8130</v>
-      </c>
+      <c r="D154" s="2" t="inlineStr"/>
+      <c r="E154" s="2" t="inlineStr"/>
+      <c r="F154" s="2" t="inlineStr"/>
       <c r="G154" s="2" t="inlineStr"/>
       <c r="H154" s="2" t="inlineStr"/>
     </row>
@@ -14180,19 +14050,9 @@
           <t>Postcode prefix page</t>
         </is>
       </c>
-      <c r="D155" s="3" t="inlineStr">
-        <is>
-          <t>SG1 Broadband Deals | BroadbandPicker</t>
-        </is>
-      </c>
-      <c r="E155" s="3" t="inlineStr">
-        <is>
-          <t>Best Broadband Deals in Stevenage ( SG1 )</t>
-        </is>
-      </c>
-      <c r="F155" s="3" t="n">
-        <v>8130</v>
-      </c>
+      <c r="D155" s="3" t="inlineStr"/>
+      <c r="E155" s="3" t="inlineStr"/>
+      <c r="F155" s="3" t="inlineStr"/>
       <c r="G155" s="3" t="inlineStr"/>
       <c r="H155" s="3" t="inlineStr"/>
     </row>

</xml_diff>